<commit_message>
Updates to eps-us 4.0.5 as of 1/30/26 commit #d42679f
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
+++ b/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\bldgs\BPSfDSPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\bldgs\BPSfDSPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B358AC65-4386-4D6B-A447-C59C227A0A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B439AB3-0459-4198-9F1D-163C78F4AEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7860" yWindow="1950" windowWidth="20295" windowHeight="12150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="7" r:id="rId1"/>
-    <sheet name="BPSfDSPV" sheetId="8" r:id="rId2"/>
+    <sheet name="BPSfDSPC" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,6 +52,9 @@
     <t>None needed</t>
   </si>
   <si>
+    <t>BPSfDSPC BAU Percent Subsidy for Distributed Solar PV Capacity</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Note: </t>
     </r>
@@ -63,11 +66,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">We include the 30% 25D credit included in the Inflation Reduction Act, which is phased out through 2035. </t>
+      <t>We include the 30% 25D credit included in the Inflation Reduction Act, which is phased out in 2026</t>
     </r>
-  </si>
-  <si>
-    <t>BPSfDSPC BAU Percent Subsidy for Distributed Solar PV Capacity</t>
   </si>
 </sst>
 </file>
@@ -111,18 +111,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -141,9 +138,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -181,9 +178,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -216,26 +213,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -268,26 +248,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -470,14 +433,14 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -486,7 +449,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -500,15 +463,15 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B1">
@@ -606,94 +569,94 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6">
-        <v>0</v>
-      </c>
-      <c r="C2" s="6">
-        <v>0</v>
-      </c>
-      <c r="D2" s="6">
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
         <v>0.3</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2">
         <v>0.3</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2">
         <v>0.3</v>
       </c>
-      <c r="G2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="J2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0.26</v>
-      </c>
-      <c r="O2" s="6">
-        <v>0.22</v>
-      </c>
-      <c r="P2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>0</v>
-      </c>
-      <c r="R2" s="6">
-        <v>0</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6">
-        <v>0</v>
-      </c>
-      <c r="U2" s="6">
-        <v>0</v>
-      </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="6">
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
         <v>0</v>
       </c>
     </row>
@@ -701,94 +664,94 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6">
-        <v>0</v>
-      </c>
-      <c r="C3" s="6">
-        <v>0</v>
-      </c>
-      <c r="D3" s="6">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>0.3</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3">
         <v>0.3</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3">
         <v>0.3</v>
       </c>
-      <c r="G3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="H3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="J3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="K3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="L3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="M3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="N3" s="6">
-        <v>0.26</v>
-      </c>
-      <c r="O3" s="6">
-        <v>0.22</v>
-      </c>
-      <c r="P3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="6">
-        <v>0</v>
-      </c>
-      <c r="R3" s="6">
-        <v>0</v>
-      </c>
-      <c r="S3" s="6">
-        <v>0</v>
-      </c>
-      <c r="T3" s="6">
-        <v>0</v>
-      </c>
-      <c r="U3" s="6">
-        <v>0</v>
-      </c>
-      <c r="V3" s="6">
-        <v>0</v>
-      </c>
-      <c r="W3" s="6">
-        <v>0</v>
-      </c>
-      <c r="X3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="6">
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
         <v>0</v>
       </c>
     </row>
@@ -796,105 +759,96 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6">
-        <v>0</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0</v>
-      </c>
-      <c r="D4" s="6">
-        <v>0</v>
-      </c>
-      <c r="E4" s="6">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>0</v>
-      </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
-        <v>0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="6">
-        <v>0</v>
-      </c>
-      <c r="N4" s="6">
-        <v>0</v>
-      </c>
-      <c r="O4" s="6">
-        <v>0</v>
-      </c>
-      <c r="P4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="6">
-        <v>0</v>
-      </c>
-      <c r="R4" s="6">
-        <v>0</v>
-      </c>
-      <c r="S4" s="6">
-        <v>0</v>
-      </c>
-      <c r="T4" s="6">
-        <v>0</v>
-      </c>
-      <c r="U4" s="6">
-        <v>0</v>
-      </c>
-      <c r="V4" s="6">
-        <v>0</v>
-      </c>
-      <c r="W4" s="6">
-        <v>0</v>
-      </c>
-      <c r="X4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="B5" s="3"/>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update to most recent eps-us develop commit
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
+++ b/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26327"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\bldgs\BPSfDSPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\bldgs\BPSfDSPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B439AB3-0459-4198-9F1D-163C78F4AEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B358AC65-4386-4D6B-A447-C59C227A0A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7860" yWindow="1950" windowWidth="20295" windowHeight="12150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="7" r:id="rId1"/>
-    <sheet name="BPSfDSPC" sheetId="8" r:id="rId2"/>
+    <sheet name="BPSfDSPV" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,9 +52,6 @@
     <t>None needed</t>
   </si>
   <si>
-    <t>BPSfDSPC BAU Percent Subsidy for Distributed Solar PV Capacity</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Note: </t>
     </r>
@@ -66,8 +63,11 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>We include the 30% 25D credit included in the Inflation Reduction Act, which is phased out in 2026</t>
+      <t xml:space="preserve">We include the 30% 25D credit included in the Inflation Reduction Act, which is phased out through 2035. </t>
     </r>
+  </si>
+  <si>
+    <t>BPSfDSPC BAU Percent Subsidy for Distributed Solar PV Capacity</t>
   </si>
 </sst>
 </file>
@@ -111,15 +111,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -138,9 +141,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -178,9 +181,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -213,9 +216,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -248,9 +268,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -433,14 +470,14 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -449,7 +486,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -463,15 +500,15 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B1">
@@ -569,94 +606,94 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0.3</v>
-      </c>
-      <c r="E2">
-        <v>0.3</v>
-      </c>
-      <c r="F2">
-        <v>0.3</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
-      </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-      <c r="X2">
-        <v>0</v>
-      </c>
-      <c r="Y2">
-        <v>0</v>
-      </c>
-      <c r="Z2">
-        <v>0</v>
-      </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-      <c r="AC2">
-        <v>0</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2">
+      <c r="B2" s="6">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6">
+        <v>0</v>
+      </c>
+      <c r="D2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="E2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="F2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="G2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="H2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="I2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="J2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="K2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="L2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="M2" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="N2" s="6">
+        <v>0.26</v>
+      </c>
+      <c r="O2" s="6">
+        <v>0.22</v>
+      </c>
+      <c r="P2" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="6">
+        <v>0</v>
+      </c>
+      <c r="R2" s="6">
+        <v>0</v>
+      </c>
+      <c r="S2" s="6">
+        <v>0</v>
+      </c>
+      <c r="T2" s="6">
+        <v>0</v>
+      </c>
+      <c r="U2" s="6">
+        <v>0</v>
+      </c>
+      <c r="V2" s="6">
+        <v>0</v>
+      </c>
+      <c r="W2" s="6">
+        <v>0</v>
+      </c>
+      <c r="X2" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="6">
         <v>0</v>
       </c>
     </row>
@@ -664,94 +701,94 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0.3</v>
-      </c>
-      <c r="E3">
-        <v>0.3</v>
-      </c>
-      <c r="F3">
-        <v>0.3</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3">
-        <v>0</v>
-      </c>
-      <c r="U3">
-        <v>0</v>
-      </c>
-      <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <v>0</v>
-      </c>
-      <c r="X3">
-        <v>0</v>
-      </c>
-      <c r="Y3">
-        <v>0</v>
-      </c>
-      <c r="Z3">
-        <v>0</v>
-      </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AB3">
-        <v>0</v>
-      </c>
-      <c r="AC3">
-        <v>0</v>
-      </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
-      <c r="AE3">
+      <c r="B3" s="6">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="G3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="H3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="I3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="J3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="K3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="L3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="M3" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="N3" s="6">
+        <v>0.26</v>
+      </c>
+      <c r="O3" s="6">
+        <v>0.22</v>
+      </c>
+      <c r="P3" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="6">
+        <v>0</v>
+      </c>
+      <c r="R3" s="6">
+        <v>0</v>
+      </c>
+      <c r="S3" s="6">
+        <v>0</v>
+      </c>
+      <c r="T3" s="6">
+        <v>0</v>
+      </c>
+      <c r="U3" s="6">
+        <v>0</v>
+      </c>
+      <c r="V3" s="6">
+        <v>0</v>
+      </c>
+      <c r="W3" s="6">
+        <v>0</v>
+      </c>
+      <c r="X3" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="6">
         <v>0</v>
       </c>
     </row>
@@ -759,96 +796,105 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4">
-        <v>0</v>
-      </c>
-      <c r="U4">
-        <v>0</v>
-      </c>
-      <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-      <c r="X4">
-        <v>0</v>
-      </c>
-      <c r="Y4">
-        <v>0</v>
-      </c>
-      <c r="Z4">
-        <v>0</v>
-      </c>
-      <c r="AA4">
-        <v>0</v>
-      </c>
-      <c r="AB4">
-        <v>0</v>
-      </c>
-      <c r="AC4">
-        <v>0</v>
-      </c>
-      <c r="AD4">
-        <v>0</v>
-      </c>
-      <c r="AE4">
-        <v>0</v>
-      </c>
+      <c r="B4" s="6">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0</v>
+      </c>
+      <c r="D4" s="6">
+        <v>0</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6">
+        <v>0</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>0</v>
+      </c>
+      <c r="I4" s="6">
+        <v>0</v>
+      </c>
+      <c r="J4" s="6">
+        <v>0</v>
+      </c>
+      <c r="K4" s="6">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6">
+        <v>0</v>
+      </c>
+      <c r="M4" s="6">
+        <v>0</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0</v>
+      </c>
+      <c r="O4" s="6">
+        <v>0</v>
+      </c>
+      <c r="P4" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="6">
+        <v>0</v>
+      </c>
+      <c r="R4" s="6">
+        <v>0</v>
+      </c>
+      <c r="S4" s="6">
+        <v>0</v>
+      </c>
+      <c r="T4" s="6">
+        <v>0</v>
+      </c>
+      <c r="U4" s="6">
+        <v>0</v>
+      </c>
+      <c r="V4" s="6">
+        <v>0</v>
+      </c>
+      <c r="W4" s="6">
+        <v>0</v>
+      </c>
+      <c r="X4" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="B7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update to most recent 4.0.5 commit
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
+++ b/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\bldgs\BPSfDSPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\bldgs\BPSfDSPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B358AC65-4386-4D6B-A447-C59C227A0A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B439AB3-0459-4198-9F1D-163C78F4AEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7860" yWindow="1950" windowWidth="20295" windowHeight="12150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="7" r:id="rId1"/>
-    <sheet name="BPSfDSPV" sheetId="8" r:id="rId2"/>
+    <sheet name="BPSfDSPC" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,6 +52,9 @@
     <t>None needed</t>
   </si>
   <si>
+    <t>BPSfDSPC BAU Percent Subsidy for Distributed Solar PV Capacity</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Note: </t>
     </r>
@@ -63,11 +66,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">We include the 30% 25D credit included in the Inflation Reduction Act, which is phased out through 2035. </t>
+      <t>We include the 30% 25D credit included in the Inflation Reduction Act, which is phased out in 2026</t>
     </r>
-  </si>
-  <si>
-    <t>BPSfDSPC BAU Percent Subsidy for Distributed Solar PV Capacity</t>
   </si>
 </sst>
 </file>
@@ -111,18 +111,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -141,9 +138,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -181,9 +178,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -216,26 +213,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -268,26 +248,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -470,14 +433,14 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -486,7 +449,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -500,15 +463,15 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B1">
@@ -606,94 +569,94 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6">
-        <v>0</v>
-      </c>
-      <c r="C2" s="6">
-        <v>0</v>
-      </c>
-      <c r="D2" s="6">
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
         <v>0.3</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2">
         <v>0.3</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2">
         <v>0.3</v>
       </c>
-      <c r="G2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="J2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0.26</v>
-      </c>
-      <c r="O2" s="6">
-        <v>0.22</v>
-      </c>
-      <c r="P2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>0</v>
-      </c>
-      <c r="R2" s="6">
-        <v>0</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6">
-        <v>0</v>
-      </c>
-      <c r="U2" s="6">
-        <v>0</v>
-      </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="6">
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
         <v>0</v>
       </c>
     </row>
@@ -701,94 +664,94 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6">
-        <v>0</v>
-      </c>
-      <c r="C3" s="6">
-        <v>0</v>
-      </c>
-      <c r="D3" s="6">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>0.3</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3">
         <v>0.3</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3">
         <v>0.3</v>
       </c>
-      <c r="G3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="H3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="J3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="K3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="L3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="M3" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="N3" s="6">
-        <v>0.26</v>
-      </c>
-      <c r="O3" s="6">
-        <v>0.22</v>
-      </c>
-      <c r="P3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="6">
-        <v>0</v>
-      </c>
-      <c r="R3" s="6">
-        <v>0</v>
-      </c>
-      <c r="S3" s="6">
-        <v>0</v>
-      </c>
-      <c r="T3" s="6">
-        <v>0</v>
-      </c>
-      <c r="U3" s="6">
-        <v>0</v>
-      </c>
-      <c r="V3" s="6">
-        <v>0</v>
-      </c>
-      <c r="W3" s="6">
-        <v>0</v>
-      </c>
-      <c r="X3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="6">
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
         <v>0</v>
       </c>
     </row>
@@ -796,105 +759,96 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6">
-        <v>0</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0</v>
-      </c>
-      <c r="D4" s="6">
-        <v>0</v>
-      </c>
-      <c r="E4" s="6">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>0</v>
-      </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
-        <v>0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="6">
-        <v>0</v>
-      </c>
-      <c r="N4" s="6">
-        <v>0</v>
-      </c>
-      <c r="O4" s="6">
-        <v>0</v>
-      </c>
-      <c r="P4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="6">
-        <v>0</v>
-      </c>
-      <c r="R4" s="6">
-        <v>0</v>
-      </c>
-      <c r="S4" s="6">
-        <v>0</v>
-      </c>
-      <c r="T4" s="6">
-        <v>0</v>
-      </c>
-      <c r="U4" s="6">
-        <v>0</v>
-      </c>
-      <c r="V4" s="6">
-        <v>0</v>
-      </c>
-      <c r="W4" s="6">
-        <v>0</v>
-      </c>
-      <c r="X4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="B5" s="3"/>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>